<commit_message>
Updating mapping tables and code to process 2024 data.
Updating mapping tables and code to process 2024 data.
</commit_message>
<xml_diff>
--- a/mappings/hoedanigheid_mapped.xlsx
+++ b/mappings/hoedanigheid_mapped.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projecten\RWS\ISC-mapping-schelde\mappings\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ocean\Work\Projects\2026\ISC\Tools\Repositories\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E8A2106-9042-4793-BD90-71754DAE090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF66827-5AA9-4377-848D-2B621DD6D27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>nf</t>
   </si>
@@ -107,6 +107,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -116,12 +117,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -151,12 +158,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -462,9 +476,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -472,7 +489,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -480,7 +497,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -488,7 +505,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -496,7 +513,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -504,15 +521,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -520,20 +537,23 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -541,12 +561,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -554,7 +574,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -562,7 +582,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -570,27 +590,33 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B15" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Updating substances in mapping table and code.
Updating substances in mapping table and code.
</commit_message>
<xml_diff>
--- a/mappings/hoedanigheid_mapped.xlsx
+++ b/mappings/hoedanigheid_mapped.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ocean\Work\Projects\2026\ISC\Tools\Repositories\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF66827-5AA9-4377-848D-2B621DD6D27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA86D9B-9D07-4436-B89A-0DD49F9425D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-45" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>nf</t>
   </si>
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -167,10 +167,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -525,7 +524,7 @@
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -541,7 +540,7 @@
       <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -549,7 +548,7 @@
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -565,12 +564,15 @@
       <c r="A11" t="s">
         <v>9</v>
       </c>
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -586,7 +588,7 @@
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
     </row>
@@ -594,7 +596,7 @@
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>21</v>
       </c>
     </row>
@@ -602,7 +604,7 @@
       <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating code addressing latest comments .
Updating code addressing latest comments .
</commit_message>
<xml_diff>
--- a/mappings/hoedanigheid_mapped.xlsx
+++ b/mappings/hoedanigheid_mapped.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ocean\Work\Projects\2026\ISC\Tools\Repositories\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA86D9B-9D07-4436-B89A-0DD49F9425D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F3EF16-CCD6-4684-8E84-51E41639DA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-45" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>nf</t>
   </si>
@@ -65,15 +65,6 @@
   </si>
   <si>
     <t>CaCO3</t>
-  </si>
-  <si>
-    <t>WATSGL</t>
-  </si>
-  <si>
-    <t>Gd</t>
-  </si>
-  <si>
-    <t>Cl</t>
   </si>
   <si>
     <t>hoedanigheid_code_wadar</t>
@@ -158,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -168,7 +159,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -474,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.109375" customWidth="1"/>
@@ -482,10 +472,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -493,7 +483,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -501,7 +491,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -509,7 +499,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -517,7 +507,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -525,7 +515,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -533,7 +523,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -541,7 +531,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -549,7 +539,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -557,7 +547,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -565,7 +555,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -573,7 +563,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -581,46 +571,31 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>22</v>
+      <c r="B14" s="4" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>21</v>
+      <c r="B15" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>17</v>
+      <c r="B16" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>